<commit_message>
L9, C455a, c455b are now set to be fitted instead of DNF. New BOM and Pick & place data generated.
</commit_message>
<xml_diff>
--- a/manufacturing/BOM/BOM_AFC_v4.0.5_DUNE.xlsx
+++ b/manufacturing/BOM/BOM_AFC_v4.0.5_DUNE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/msaleh_ic_ac_uk/Documents/Desktop/FMC CARRIER AFC/DUNE-Variant-AMC-FMC-Carrier-AFC/manufacturing/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A65342E-09EA-4172-BC26-0FCE8F93BB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D28365EF-2140-4672-BCA0-63CB1CF1A831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="270" yWindow="0" windowWidth="16410" windowHeight="13760" xr2:uid="{A163943B-4781-4035-92F2-FE78869B403A}"/>
+    <workbookView xWindow="230" yWindow="1710" windowWidth="28800" windowHeight="15290" xr2:uid="{FC3D136D-E780-40A3-A15C-B5DECDC19390}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_AFC_v4.0.5_DUNE" sheetId="1" r:id="rId1"/>
@@ -92,7 +92,7 @@
     <t>Non-polarised capacitor</t>
   </si>
   <si>
-    <t>C1A, C1B, C5A, C5B, C7A, C7B, C46, C47, C66, C68, C79, C81, C85, C87, C116, C117, C119, C122, C123, C136, C137, C139, C142, C154, C155, C156, C157, C158, C161, C162, C163, C164, C165, C168, C169, C170, C171, C172, C173, C174, C175, C176, C177, C454, C462, C464, C471, C472, C474, C477, C529, C530, C531, C534, C540, C541, C542, C544, C545, C546</t>
+    <t>C1A, C1B, C5A, C5B, C7A, C7B, C46, C47, C66, C68, C79, C81, C85, C87, C116, C117, C119, C122, C123, C136, C137, C139, C142, C154, C155, C156, C157, C158, C161, C162, C163, C164, C165, C168, C169, C170, C171, C172, C173, C174, C175, C176, C177, C454, C455a, C455b, C462, C464, C471, C472, C474, C477, C529, C530, C531, C534, C540, C541, C542, C544, C545, C546</t>
   </si>
   <si>
     <t>1206, [NoParam]</t>
@@ -1115,7 +1115,7 @@
     <t>Semi-shielded Power Inductor, 1 uH, +/- 30%, 2.35 A, -40 to 125 degC, 3 x 3 x 1.5 mm SMD, RoHS and Halogen Free, Tape and Reel</t>
   </si>
   <si>
-    <t>L2, L4, L7</t>
+    <t>L2, L4, L7, L9</t>
   </si>
   <si>
     <t>Bourns</t>
@@ -2147,7 +2147,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39E87576-E4AC-4179-A49E-4A530C7970BA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B868DF9-9DB0-4CC4-8DC6-2F143E5B60D4}">
   <dimension ref="A1:I139"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2226,7 +2226,7 @@
         <v>17</v>
       </c>
       <c r="E3" s="1">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>18</v>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="D80" s="1"/>
       <c r="E80" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>358</v>

</xml_diff>

<commit_message>
C840, C841, C202 and C203 ar now DNF. C219, C220, C399, C397, C461, C463, C838 and C839 are now fitted components.
</commit_message>
<xml_diff>
--- a/manufacturing/BOM/BOM_AFC_v4.0.5_DUNE.xlsx
+++ b/manufacturing/BOM/BOM_AFC_v4.0.5_DUNE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/msaleh_ic_ac_uk/Documents/Desktop/FMC CARRIER AFC/DUNE-Variant-AMC-FMC-Carrier-AFC/manufacturing/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D28365EF-2140-4672-BCA0-63CB1CF1A831}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB5720F2-9165-40E2-9F82-9505B8399D36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="230" yWindow="1710" windowWidth="28800" windowHeight="15290" xr2:uid="{FC3D136D-E780-40A3-A15C-B5DECDC19390}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{40C8643C-3B07-4FFB-83B8-1FF8B6554006}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_AFC_v4.0.5_DUNE" sheetId="1" r:id="rId1"/>
@@ -128,7 +128,7 @@
     <t>100nF</t>
   </si>
   <si>
-    <t>C4A, C4B, C6A, C6B, C10A, C10B, C11A, C11B, C15A, C15B, C20, C21, C22, C23, C24, C25, C26, C27, C28, C29, C30, C52, C56, C57, C58, C59, C61, C63, C65, C67, C69, C70, C73, C74, C75, C76, C78, C80, C82, C83, C84, C88, C89, C93, C94, C95, C96, C98, C99, C100, C101, C102, C103, C104, C105, C109, C110, C111, C112, C114, C118, C120, C121, C124, C125, C129, C131, C132, C134, C138, C140, C141, C178, C179, C180, C181, C182, C183, C184, C185, C186, C187, C188, C189, C190, C191, C192, C193, C194, C195, C196, C197, C198, C199, C200, C201, C202, C203, C204, C205, C206, C207, C211, C212, C213, C214, C215, C216, C217, C221, C222, C223, C224, C225, C227, C228, C255, C256, C257, C258, C262, C263, C273, C274, C281, C282, C289, C290, C297, C298, C299, C300, C301, C302, C303, C304, C305, C307, C308, C309, C310, C311, C312, C313, C314, C315, C316, C317, C334, C335, C336, C337, C338, C339, C340, C341, C342, C343, C344, C345, C346, C347, C348, C349, C350, C351, C352, C353, C354, C355, C356, C357, C358, C359, C360, C361, C362, C363, C364, C365, C366, C367, C368, C369, C370, C371, C372, C373, C374, C375, C376, C377, C378, C379, C380, C381, C382, C383, C384, C385, C386, C387, C388, C392, C393, C394, C395, C398, C400, C401, C402, C403, C404, C405, C407, C408, C409, C411, C412, C413, C414, C415, C416, C417, C418, C419, C421, C427, C434, C435, C436, C437, C438, C439, C440, C441, C443, C444, C445, C452, C455, C457, C459, C468, C476, C480, C481, C482, C483, C484, C485, C486, C487, C496, C508, C509, C510, C512, C514, C515, C516, C517, C518, C524, C548, C567, C568, C569, C574, C575, C590, C595, C604, C613, C618, C620, C624, C625, C626, C627, C628, C629, C630, C631, C632, C633, C726, C727, C728, C729, C734, C735, C736, C737, C749, C751, C752, C753, C754, C755, C756, C757, C760, C761, C762, C763, C764, C765, C766, C767, C840, C841, C847, C855</t>
+    <t>C4A, C4B, C6A, C6B, C10A, C10B, C11A, C11B, C15A, C15B, C20, C21, C22, C23, C24, C25, C26, C27, C28, C29, C30, C52, C56, C57, C58, C59, C61, C63, C65, C67, C69, C70, C73, C74, C75, C76, C78, C80, C82, C83, C84, C88, C89, C93, C94, C95, C96, C98, C99, C100, C101, C102, C103, C104, C105, C109, C110, C111, C112, C114, C118, C120, C121, C124, C125, C129, C131, C132, C134, C138, C140, C141, C178, C179, C180, C181, C182, C183, C184, C185, C186, C187, C188, C189, C190, C191, C192, C193, C194, C195, C196, C197, C198, C199, C200, C201, C204, C205, C206, C207, C211, C212, C213, C214, C215, C216, C217, C219, C220, C221, C222, C223, C224, C225, C227, C228, C255, C256, C257, C258, C262, C263, C273, C274, C281, C282, C289, C290, C297, C298, C299, C300, C301, C302, C303, C304, C305, C307, C308, C309, C310, C311, C312, C313, C314, C315, C316, C317, C334, C335, C336, C337, C338, C339, C340, C341, C342, C343, C344, C345, C346, C347, C348, C349, C350, C351, C352, C353, C354, C355, C356, C357, C358, C359, C360, C361, C362, C363, C364, C365, C366, C367, C368, C369, C370, C371, C372, C373, C374, C375, C376, C377, C378, C379, C380, C381, C382, C383, C384, C385, C386, C387, C388, C392, C393, C394, C395, C397, C398, C399, C400, C401, C402, C403, C404, C405, C407, C408, C409, C411, C412, C413, C414, C415, C416, C417, C418, C419, C421, C427, C434, C435, C436, C437, C438, C439, C440, C441, C443, C444, C445, C452, C455, C457, C459, C461, C463, C468, C476, C480, C481, C482, C483, C484, C485, C486, C487, C496, C508, C509, C510, C512, C514, C515, C516, C517, C518, C524, C548, C567, C568, C569, C574, C575, C590, C595, C604, C613, C618, C620, C624, C625, C626, C627, C628, C629, C630, C631, C632, C633, C726, C727, C728, C729, C734, C735, C736, C737, C749, C751, C752, C753, C754, C755, C756, C757, C760, C761, C762, C763, C764, C765, C766, C767, C838, C839, C847, C855</t>
   </si>
   <si>
     <t>0201</t>
@@ -2147,7 +2147,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B868DF9-9DB0-4CC4-8DC6-2F143E5B60D4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D52A0302-AB38-4DC6-B1AE-25FE9239973A}">
   <dimension ref="A1:I139"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2284,7 +2284,7 @@
         <v>29</v>
       </c>
       <c r="E5" s="1">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>18</v>

</xml_diff>